<commit_message>
feat: historic data pipeline, load:historic script, V2 auto-calibration (system_settings), dashboard fixes
- Add load:historic script and pnpm load:historic (latest/specific/--all)
- Add system_settings table (00016), calibration_v2 seed, RLS
- Add calibration-service (recalculateCalibration, refreshCalibrationCache), calibration-cache
- Classifier: read calibration from cache (DB) then file then HISTORICAL_CALIBRATION
- Sync route: auto-run recalculateCalibration after tender upsert (zero-touch)
- Evaluation action: refreshCalibrationCache before scoring
- Add calibrate-from-db script (optional one-off), calibrate:from-db pnpm script
- RUNBOOK + DATA_PIPELINE_HISTORIC_AND_V2 docs, types/database system_settings

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/Odoo_Leads_Import.xlsx
+++ b/output/Odoo_Leads_Import.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I51"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,33 +430,33 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>High-value IT infrastructure project</v>
+        <v>توريد وتركيب وتكامل أجهزة «بنان» لنظام التحقق من الهوية بمستشفى الإمام عبد الرحمن آل فيصل بالدمام التابع للشؤون الصحية بوزارة الحرس الوطني</v>
       </c>
       <c r="B2" t="str">
-        <v>Test Government Entity</v>
-      </c>
-      <c r="C2">
-        <v>5000000</v>
+        <v>الشؤون الصحیة بوزارة الحرس الوطني</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>2026-03-15T23:59:59.999Z</v>
+        <v>2099-12-31T00:00:00.000Z</v>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Tender Number: TEST001
-Score: 97 | Recommendation: Pursue
-- Estimated value in range
-- 43 days until deadline
+        <v xml:space="preserve">Tender Number: 260139009288
+Score: 75 | Recommendation: Pursue
+- No estimated value
+- 26995 days until deadline
 - Low cost of entry
 - Title and description present</v>
       </c>
       <c r="F2">
-        <v>97</v>
+        <v>75</v>
       </c>
       <c r="G2" t="str">
         <v>Pursue</v>
       </c>
       <c r="H2" t="str">
-        <v>TEST001</v>
+        <v>260139009288</v>
       </c>
       <c r="I2" t="str">
         <v>etimad</v>
@@ -464,32 +464,32 @@
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3" t="str">
-        <v>Small IT support contract</v>
+        <v>مركز المراقبة والتحكم وتشغيل حلول الصحة الرقمية للخدمات الطبية العسكرية</v>
       </c>
       <c r="B3" t="str">
-        <v>Test Agency</v>
-      </c>
-      <c r="C3">
-        <v>50000</v>
+        <v>رئاسة هيئة الأركان العامة</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
       </c>
       <c r="D3" t="str">
-        <v>2026-01-25T23:59:59.999Z</v>
+        <v>2026-03-27T00:00:00.000Z</v>
       </c>
       <c r="E3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Tender Number: TEST003
-Score: 73 | Recommendation: Pursue
-- Estimated value in range
-- Deadline passed
+        <v xml:space="preserve">Tender Number: 250939014491
+Score: 55 | Recommendation: Monitor
+- No estimated value
+- 53 days until deadline
 - Title and description present</v>
       </c>
       <c r="F3">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="G3" t="str">
-        <v>Pursue</v>
+        <v>Monitor</v>
       </c>
       <c r="H3" t="str">
-        <v>TEST003</v>
+        <v>250939014491</v>
       </c>
       <c r="I3" t="str">
         <v>etimad</v>
@@ -497,40 +497,1591 @@
     </row>
     <row r="4" xml:space="preserve">
       <c r="A4" t="str">
-        <v>Medium-value software development</v>
+        <v>مشروع الدعم الفني للانظمة المفتوحة - المرحلة الرابعة</v>
       </c>
       <c r="B4" t="str">
-        <v>Test Ministry</v>
-      </c>
-      <c r="C4">
-        <v>500000</v>
+        <v>الهيئة السعودية للبيانات والذكاء الاصطناعي</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
       </c>
       <c r="D4" t="str">
-        <v>2026-02-10T23:59:59.999Z</v>
+        <v>2026-03-29T00:00:00.000Z</v>
       </c>
       <c r="E4" t="str" xml:space="preserve">
-        <v xml:space="preserve">Tender Number: TEST002
-Score: 60 | Recommendation: Monitor
-- Estimated value in range
+        <v xml:space="preserve">Tender Number: 251239002892
+Score: 55 | Recommendation: Monitor
+- No estimated value
+- 55 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F4">
+        <v>55</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H4" t="str">
+        <v>251239002892</v>
+      </c>
+      <c r="I4" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>تشغيل مراكز الاتصال وزارة الصحة</v>
+      </c>
+      <c r="B5" t="str">
+        <v>وزارة الصحة الديوان العام</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v>2026-03-29T00:00:00.000Z</v>
+      </c>
+      <c r="E5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 251239009414
+Score: 55 | Recommendation: Monitor
+- No estimated value
+- 55 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F5">
+        <v>55</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H5" t="str">
+        <v>251239009414</v>
+      </c>
+      <c r="I5" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>فحص واختبار وتجهيز البنية الرقمية للمباني الإدارية والمراكز الاسعافية لموسم الحج 1447هـ</v>
+      </c>
+      <c r="B6" t="str">
+        <v>هيئة الهلال الأحمر السعودي</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v>2099-12-31T00:00:00.000Z</v>
+      </c>
+      <c r="E6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139005166
+Score: 55 | Recommendation: Monitor
+- No estimated value
+- 26995 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F6">
+        <v>55</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H6" t="str">
+        <v>260139005166</v>
+      </c>
+      <c r="I6" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>تجديد الدعم لأنظمة ساب</v>
+      </c>
+      <c r="B7" t="str">
+        <v>صندوق التنمية الصناعية</v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>2026-03-01T00:00:00.000Z</v>
+      </c>
+      <c r="E7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139004525
+Score: 52 | Recommendation: Monitor
+- No estimated value
+- 27 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F7">
+        <v>52</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H7" t="str">
+        <v>260139004525</v>
+      </c>
+      <c r="I7" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>مشروع تحديث الشبكات (الهاتفية –الانترنت –التلفزيونية) بمنطقة الرياض</v>
+      </c>
+      <c r="B8" t="str">
+        <v>المباحث العامة</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v>2026-02-22T00:00:00.000Z</v>
+      </c>
+      <c r="E8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139005990
+Score: 50 | Recommendation: Monitor
+- No estimated value
+- 20 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F8">
+        <v>50</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H8" t="str">
+        <v>260139005990</v>
+      </c>
+      <c r="I8" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>MEDICAL CART STYLI VIEW SV10</v>
+      </c>
+      <c r="B9" t="str">
+        <v>مستشفى مجمع الملك فهد الطبي بالظهران</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v>2026-02-09T00:00:00.000Z</v>
+      </c>
+      <c r="E9" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139008862
+Score: 50 | Recommendation: Monitor
+- No estimated value
+- 7 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F9">
+        <v>50</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H9" t="str">
+        <v>260139008862</v>
+      </c>
+      <c r="I9" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>مشروع تشغيل وصيانة الخدمات الالكترونية لوكالة تنمية المجتمع</v>
+      </c>
+      <c r="B10" t="str">
+        <v>وزارة الموارد البشرية والتنمية الاجتماعية</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v>2026-02-26T00:00:00.000Z</v>
+      </c>
+      <c r="E10" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139006813
+Score: 48 | Recommendation: Monitor
+- No estimated value
+- 24 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F10">
+        <v>48</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H10" t="str">
+        <v>260139006813</v>
+      </c>
+      <c r="I10" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>تجديد الرخص والدعم لنظام تيراداتا</v>
+      </c>
+      <c r="B11" t="str">
+        <v>هيئة الزكاة والضريبة والجمارك</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v>2026-02-27T00:00:00.000Z</v>
+      </c>
+      <c r="E11" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139005549
+Score: 47 | Recommendation: Monitor
+- No estimated value
+- 25 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F11">
+        <v>47</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H11" t="str">
+        <v>260139005549</v>
+      </c>
+      <c r="I11" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>تجديد رخص تطبيق ( adobe creative cloud ) و تطبيق (adobe acrobat pro ) وتوريد رخص تطبيق ( shutterstock) (Motion array) (Envato elaments)-(freepik)- (Canva Pro) أو ما يعادلها</v>
+      </c>
+      <c r="B12" t="str">
+        <v>حرس الحدود - التقنية والذكاء الاصطناعي</v>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v>2026-02-03T00:00:00.000Z</v>
+      </c>
+      <c r="E12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139006991
+Score: 47 | Recommendation: Monitor
+- No estimated value
+- 1 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F12">
+        <v>47</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H12" t="str">
+        <v>260139006991</v>
+      </c>
+      <c r="I12" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>تجديد اشتراك بخدمة مقيم</v>
+      </c>
+      <c r="B13" t="str">
+        <v>بلدية محافظة تيماء</v>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v>2026-02-04T00:00:00.000Z</v>
+      </c>
+      <c r="E13" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139009338
+Score: 47 | Recommendation: Monitor
+- No estimated value
+- 2 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F13">
+        <v>47</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H13" t="str">
+        <v>260139009338</v>
+      </c>
+      <c r="I13" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>خدمات احترافية لضبط اختبارات الجودة للمشاريع والتحسينات التقنية</v>
+      </c>
+      <c r="B14" t="str">
+        <v>هيئة السوق المالية</v>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v>2026-02-15T00:00:00.000Z</v>
+      </c>
+      <c r="E14" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139009423
+Score: 47 | Recommendation: Monitor
+- No estimated value
+- 13 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F14">
+        <v>47</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H14" t="str">
+        <v>260139009423</v>
+      </c>
+      <c r="I14" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>تأمين احتياجات إدارة التواصل في الإدارة التنفيذية العليا لتجمع جدة الصحي الثاني</v>
+      </c>
+      <c r="B15" t="str">
+        <v>تجمع جدة الصحي الثاني</v>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v>2026-02-04T00:00:00.000Z</v>
+      </c>
+      <c r="E15" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139009968
+Score: 47 | Recommendation: Monitor
+- No estimated value
+- 2 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F15">
+        <v>47</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H15" t="str">
+        <v>260139009968</v>
+      </c>
+      <c r="I15" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>تامين رخصة برامج لوكالة الوزارة لشؤون الدعوة والارشاد لإدارة الدعوة الرقمية</v>
+      </c>
+      <c r="B16" t="str">
+        <v>وزارة الشـؤون الاسلامية والدعوة والارشاد</v>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v>2026-02-01T00:00:00.000Z</v>
+      </c>
+      <c r="E16" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 251039019624
+Score: 46 | Recommendation: Monitor
+- No estimated value
+- Deadline passed
+- Title and description present</v>
+      </c>
+      <c r="F16">
+        <v>46</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H16" t="str">
+        <v>251039019624</v>
+      </c>
+      <c r="I16" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>احتياج مشروع الخدمة الذاتية والنداء الالي للعيادات الخارجية بمستشفى الثغر العام بجدة</v>
+      </c>
+      <c r="B17" t="str">
+        <v>تجمع جدة الصحي الاول</v>
+      </c>
+      <c r="C17" t="str">
+        <v/>
+      </c>
+      <c r="D17" t="str">
+        <v>2026-02-02T00:00:00.000Z</v>
+      </c>
+      <c r="E17" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139007088
+Score: 46 | Recommendation: Monitor
+- No estimated value
+- 0 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F17">
+        <v>46</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H17" t="str">
+        <v>260139007088</v>
+      </c>
+      <c r="I17" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>توريد احبار لبعض الطابعات بادارة الشؤون الفنية المركزية بمنطقة حائل</v>
+      </c>
+      <c r="B18" t="str">
+        <v>ادارة الشؤون الفنية المركزية بمنطقة حائل</v>
+      </c>
+      <c r="C18" t="str">
+        <v/>
+      </c>
+      <c r="D18" t="str">
+        <v>2026-02-02T00:00:00.000Z</v>
+      </c>
+      <c r="E18" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139008023
+Score: 46 | Recommendation: Monitor
+- No estimated value
+- 0 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F18">
+        <v>46</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H18" t="str">
+        <v>260139008023</v>
+      </c>
+      <c r="I18" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>توفير اشتراك كاشف الاستلال العلمي iThenticate</v>
+      </c>
+      <c r="B19" t="str">
+        <v>الجامعة السعودية الالكترونية</v>
+      </c>
+      <c r="C19" t="str">
+        <v/>
+      </c>
+      <c r="D19" t="str">
+        <v>2026-02-01T00:00:00.000Z</v>
+      </c>
+      <c r="E19" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139008844
+Score: 46 | Recommendation: Monitor
+- No estimated value
+- Deadline passed
+- Title and description present</v>
+      </c>
+      <c r="F19">
+        <v>46</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H19" t="str">
+        <v>260139008844</v>
+      </c>
+      <c r="I19" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>مشروع تشغيل وصيانة وتطوير تطبيب السكتات الدماغية عن بعد</v>
+      </c>
+      <c r="B20" t="str">
+        <v>وزارة الصحة الديوان العام</v>
+      </c>
+      <c r="C20" t="str">
+        <v/>
+      </c>
+      <c r="D20" t="str">
+        <v>2026-03-01T00:00:00.000Z</v>
+      </c>
+      <c r="E20" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139002652
+Score: 44 | Recommendation: Monitor
+- No estimated value
+- 27 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F20">
+        <v>44</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H20" t="str">
+        <v>260139002652</v>
+      </c>
+      <c r="I20" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>رخص وأنظمة الأمن السيبراني</v>
+      </c>
+      <c r="B21" t="str">
+        <v>هيئة تطوير منطقة المدينة المنورة</v>
+      </c>
+      <c r="C21" t="str">
+        <v/>
+      </c>
+      <c r="D21" t="str">
+        <v>2026-02-22T00:00:00.000Z</v>
+      </c>
+      <c r="E21" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139004682
+Score: 44 | Recommendation: Monitor
+- No estimated value
+- 20 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F21">
+        <v>44</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H21" t="str">
+        <v>260139004682</v>
+      </c>
+      <c r="I21" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>مشروع تطوير وتنفيذ نظام أتمته جميع الإجراءات الداخلية والخارجية لمركز الملك عبدالعزيز للخيل العربية الأصيلة</v>
+      </c>
+      <c r="B22" t="str">
+        <v>مركز الملك عبدالعزيز للخيل العربية الأصيلة</v>
+      </c>
+      <c r="C22" t="str">
+        <v/>
+      </c>
+      <c r="D22" t="str">
+        <v>2026-03-02T00:00:00.000Z</v>
+      </c>
+      <c r="E22" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139010187
+Score: 44 | Recommendation: Monitor
+- No estimated value
+- 28 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F22">
+        <v>44</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H22" t="str">
+        <v>260139010187</v>
+      </c>
+      <c r="I22" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>توريد وتجديد رخص التطبيقات في هيئة الصحة العامة</v>
+      </c>
+      <c r="B23" t="str">
+        <v>هيئة الصحة العامة</v>
+      </c>
+      <c r="C23" t="str">
+        <v/>
+      </c>
+      <c r="D23" t="str">
+        <v>2026-02-27T00:00:00.000Z</v>
+      </c>
+      <c r="E23" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139005804
+Score: 43 | Recommendation: Monitor
+- No estimated value
+- 25 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F23">
+        <v>43</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H23" t="str">
+        <v>260139005804</v>
+      </c>
+      <c r="I23" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>تجديد الرخص والدعم الفني لنظام AppDynamics</v>
+      </c>
+      <c r="B24" t="str">
+        <v>هيئة الزكاة والضريبة والجمارك</v>
+      </c>
+      <c r="C24" t="str">
+        <v/>
+      </c>
+      <c r="D24" t="str">
+        <v>2026-02-27T00:00:00.000Z</v>
+      </c>
+      <c r="E24" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139007698
+Score: 43 | Recommendation: Monitor
+- No estimated value
+- 25 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F24">
+        <v>43</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H24" t="str">
+        <v>260139007698</v>
+      </c>
+      <c r="I24" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>تشغيل وصيانة الأمن السيبراني</v>
+      </c>
+      <c r="B25" t="str">
+        <v>أمانة منطقة حائل</v>
+      </c>
+      <c r="C25" t="str">
+        <v/>
+      </c>
+      <c r="D25" t="str">
+        <v>2026-02-27T00:00:00.000Z</v>
+      </c>
+      <c r="E25" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139008333
+Score: 43 | Recommendation: Monitor
+- No estimated value
+- 25 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F25">
+        <v>43</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H25" t="str">
+        <v>260139008333</v>
+      </c>
+      <c r="I25" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>تفعيل وبناء نماذج الدفع وشراء الخدمات الصحية المرحلة الثانية</v>
+      </c>
+      <c r="B26" t="str">
+        <v>مركز التأمين الصحي الوطني</v>
+      </c>
+      <c r="C26" t="str">
+        <v/>
+      </c>
+      <c r="D26" t="str">
+        <v>2026-02-26T00:00:00.000Z</v>
+      </c>
+      <c r="E26" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 251039001722
+Score: 42 | Recommendation: Monitor
+- No estimated value
+- 24 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F26">
+        <v>42</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H26" t="str">
+        <v>251039001722</v>
+      </c>
+      <c r="I26" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
+        <v>استضافة وتدريب النماذج اللغوية الضخمة</v>
+      </c>
+      <c r="B27" t="str">
+        <v>الهيئة السعودية للبيانات والذكاء الاصطناعي</v>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v>2026-02-26T00:00:00.000Z</v>
+      </c>
+      <c r="E27" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 251239005316
+Score: 42 | Recommendation: Monitor
+- No estimated value
+- 24 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F27">
+        <v>42</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H27" t="str">
+        <v>251239005316</v>
+      </c>
+      <c r="I27" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
+        <v>الخدمات المدارة لتشغيل وصيانة منظومة أعمال تقنية المعلومات والذكاء الاصطناعي بالأمن العام</v>
+      </c>
+      <c r="B28" t="str">
+        <v>الأمن العام (التقنية والذكاء الاصطناعي)</v>
+      </c>
+      <c r="C28" t="str">
+        <v/>
+      </c>
+      <c r="D28" t="str">
+        <v>2026-02-26T00:00:00.000Z</v>
+      </c>
+      <c r="E28" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 251239009333
+Score: 42 | Recommendation: Monitor
+- No estimated value
+- 24 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F28">
+        <v>42</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H28" t="str">
+        <v>251239009333</v>
+      </c>
+      <c r="I28" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
+        <v>الخدمات المدارة للتحول الرقمي بالجامعة السعودية الالكترونية</v>
+      </c>
+      <c r="B29" t="str">
+        <v>الجامعة السعودية الالكترونية</v>
+      </c>
+      <c r="C29" t="str">
+        <v/>
+      </c>
+      <c r="D29" t="str">
+        <v>2026-02-25T00:00:00.000Z</v>
+      </c>
+      <c r="E29" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139006263
+Score: 42 | Recommendation: Monitor
+- No estimated value
+- 23 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F29">
+        <v>42</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H29" t="str">
+        <v>260139006263</v>
+      </c>
+      <c r="I29" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30" t="str">
+        <v>مشروع أدوات البنية المؤسسية</v>
+      </c>
+      <c r="B30" t="str">
+        <v>هيئة الصحة العامة</v>
+      </c>
+      <c r="C30" t="str">
+        <v/>
+      </c>
+      <c r="D30" t="str">
+        <v>2026-02-13T00:00:00.000Z</v>
+      </c>
+      <c r="E30" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139008237
+Score: 42 | Recommendation: Monitor
+- No estimated value
+- 11 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F30">
+        <v>42</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H30" t="str">
+        <v>260139008237</v>
+      </c>
+      <c r="I30" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
+      <c r="A31" t="str">
+        <v>مشروع البوابة المعرفية لمدة 3 سنوات</v>
+      </c>
+      <c r="B31" t="str">
+        <v>جامعة الملك عبدالعزيز</v>
+      </c>
+      <c r="C31" t="str">
+        <v/>
+      </c>
+      <c r="D31" t="str">
+        <v>2026-02-12T00:00:00.000Z</v>
+      </c>
+      <c r="E31" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 251239005891
+Score: 41 | Recommendation: Monitor
+- No estimated value
 - 10 days until deadline
 - Title and description present</v>
       </c>
-      <c r="F4">
-        <v>60</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Monitor</v>
-      </c>
-      <c r="H4" t="str">
-        <v>TEST002</v>
-      </c>
-      <c r="I4" t="str">
+      <c r="F31">
+        <v>41</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H31" t="str">
+        <v>251239005891</v>
+      </c>
+      <c r="I31" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
+        <v>دعم وصيانة الأنظمة المركزية-4</v>
+      </c>
+      <c r="B32" t="str">
+        <v>الهيئة السعودية للبيانات والذكاء الاصطناعي</v>
+      </c>
+      <c r="C32" t="str">
+        <v/>
+      </c>
+      <c r="D32" t="str">
+        <v>2026-02-22T00:00:00.000Z</v>
+      </c>
+      <c r="E32" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 251139009268
+Score: 40 | Recommendation: Monitor
+- No estimated value
+- 20 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F32">
+        <v>40</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H32" t="str">
+        <v>251139009268</v>
+      </c>
+      <c r="I32" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="33" xml:space="preserve">
+      <c r="A33" t="str">
+        <v>تجديد الدعم لنظام ايراد 2026</v>
+      </c>
+      <c r="B33" t="str">
+        <v>هيئة الزكاة والضريبة والجمارك</v>
+      </c>
+      <c r="C33" t="str">
+        <v/>
+      </c>
+      <c r="D33" t="str">
+        <v>2026-02-22T00:00:00.000Z</v>
+      </c>
+      <c r="E33" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139005268
+Score: 40 | Recommendation: Monitor
+- No estimated value
+- 20 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F33">
+        <v>40</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="H33" t="str">
+        <v>260139005268</v>
+      </c>
+      <c r="I33" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="34" xml:space="preserve">
+      <c r="A34" t="str">
+        <v>تقديم خدمات تشغيل وصيانة العتاد التقني بالهيئة العامة لعقارات الدولة</v>
+      </c>
+      <c r="B34" t="str">
+        <v>الهيئة العامة لعقارات الدولة</v>
+      </c>
+      <c r="C34" t="str">
+        <v/>
+      </c>
+      <c r="D34" t="str">
+        <v>2026-02-20T00:00:00.000Z</v>
+      </c>
+      <c r="E34" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139001606
+Score: 39 | Recommendation: Ignore
+- No estimated value
+- 18 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F34">
+        <v>39</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H34" t="str">
+        <v>260139001606</v>
+      </c>
+      <c r="I34" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="35" xml:space="preserve">
+      <c r="A35" t="str">
+        <v>توريد و تشغيل جهاز بنان (جهاز التحقق من الشخصية بالبصمة) لتجمع المدينة المنورة الصحي</v>
+      </c>
+      <c r="B35" t="str">
+        <v>تجمع المدينة المنورة الصحي</v>
+      </c>
+      <c r="C35" t="str">
+        <v/>
+      </c>
+      <c r="D35" t="str">
+        <v>2026-02-11T00:00:00.000Z</v>
+      </c>
+      <c r="E35" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139003250
+Score: 39 | Recommendation: Ignore
+- No estimated value
+- 9 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F35">
+        <v>39</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H35" t="str">
+        <v>260139003250</v>
+      </c>
+      <c r="I35" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="36" xml:space="preserve">
+      <c r="A36" t="str">
+        <v>توفير رخص البرامج التعليمية المطلوبة في الكليات عبر تقنية VDI</v>
+      </c>
+      <c r="B36" t="str">
+        <v>جامعة القصيم</v>
+      </c>
+      <c r="C36" t="str">
+        <v/>
+      </c>
+      <c r="D36" t="str">
+        <v>2026-02-07T00:00:00.000Z</v>
+      </c>
+      <c r="E36" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139006779
+Score: 39 | Recommendation: Ignore
+- No estimated value
+- 5 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F36">
+        <v>39</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H36" t="str">
+        <v>260139006779</v>
+      </c>
+      <c r="I36" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="37" xml:space="preserve">
+      <c r="A37" t="str">
+        <v>تطوير وتنفيذ منصة للإبلاغ عن المخالفات</v>
+      </c>
+      <c r="B37" t="str">
+        <v>هيئة الزكاة والضريبة والجمارك</v>
+      </c>
+      <c r="C37" t="str">
+        <v/>
+      </c>
+      <c r="D37" t="str">
+        <v>2026-02-11T00:00:00.000Z</v>
+      </c>
+      <c r="E37" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139007847
+Score: 39 | Recommendation: Ignore
+- No estimated value
+- 9 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F37">
+        <v>39</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H37" t="str">
+        <v>260139007847</v>
+      </c>
+      <c r="I37" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="38" xml:space="preserve">
+      <c r="A38" t="str">
+        <v>استبدال أنظمة الحماية والتحكم الحالية بأنظمة Microsoft E5 وتفعيلها</v>
+      </c>
+      <c r="B38" t="str">
+        <v>وزارة الاستثمار</v>
+      </c>
+      <c r="C38" t="str">
+        <v/>
+      </c>
+      <c r="D38" t="str">
+        <v>2026-02-06T00:00:00.000Z</v>
+      </c>
+      <c r="E38" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139001546
+Score: 38 | Recommendation: Ignore
+- No estimated value
+- 4 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F38">
+        <v>38</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H38" t="str">
+        <v>260139001546</v>
+      </c>
+      <c r="I38" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="39" xml:space="preserve">
+      <c r="A39" t="str">
+        <v>توفير خدمات الطابعات للهيئة</v>
+      </c>
+      <c r="B39" t="str">
+        <v>هيئة تنمية الصادرات السعودية</v>
+      </c>
+      <c r="C39" t="str">
+        <v/>
+      </c>
+      <c r="D39" t="str">
+        <v>2026-02-08T00:00:00.000Z</v>
+      </c>
+      <c r="E39" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139005357
+Score: 37 | Recommendation: Ignore
+- No estimated value
+- 6 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F39">
+        <v>37</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H39" t="str">
+        <v>260139005357</v>
+      </c>
+      <c r="I39" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="40" xml:space="preserve">
+      <c r="A40" t="str">
+        <v>توريد وتركيب نظام التحكم بالتكييف والإضاءة (BMS)، بالمركز الرئيسي</v>
+      </c>
+      <c r="B40" t="str">
+        <v>الهيئة السعودية للمياه</v>
+      </c>
+      <c r="C40" t="str">
+        <v/>
+      </c>
+      <c r="D40" t="str">
+        <v>2026-02-11T00:00:00.000Z</v>
+      </c>
+      <c r="E40" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139005919
+Score: 35 | Recommendation: Ignore
+- No estimated value
+- 9 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F40">
+        <v>35</v>
+      </c>
+      <c r="G40" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H40" t="str">
+        <v>260139005919</v>
+      </c>
+      <c r="I40" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="41" xml:space="preserve">
+      <c r="A41" t="str">
+        <v>توريد أجهزة محمولة لمكتب المواءمة المالية بالديوان الملكي</v>
+      </c>
+      <c r="B41" t="str">
+        <v>برنامج الخدمات المشتركة</v>
+      </c>
+      <c r="C41" t="str">
+        <v/>
+      </c>
+      <c r="D41" t="str">
+        <v>2026-02-11T00:00:00.000Z</v>
+      </c>
+      <c r="E41" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139007772
+Score: 35 | Recommendation: Ignore
+- No estimated value
+- 9 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F41">
+        <v>35</v>
+      </c>
+      <c r="G41" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H41" t="str">
+        <v>260139007772</v>
+      </c>
+      <c r="I41" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="42" xml:space="preserve">
+      <c r="A42" t="str">
+        <v>توريد وتركيب بطاريات إضافية "UPS" لمكتب المواءمة المالية بالديوان الملكي</v>
+      </c>
+      <c r="B42" t="str">
+        <v>برنامج الخدمات المشتركة</v>
+      </c>
+      <c r="C42" t="str">
+        <v/>
+      </c>
+      <c r="D42" t="str">
+        <v>2026-02-11T00:00:00.000Z</v>
+      </c>
+      <c r="E42" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139007796
+Score: 35 | Recommendation: Ignore
+- No estimated value
+- 9 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F42">
+        <v>35</v>
+      </c>
+      <c r="G42" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H42" t="str">
+        <v>260139007796</v>
+      </c>
+      <c r="I42" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="43" xml:space="preserve">
+      <c r="A43" t="str">
+        <v>تجديد الاشتراك لمنصة الموارد البشرية</v>
+      </c>
+      <c r="B43" t="str">
+        <v>المركز الوطني لقياس أداء الأجهزة العامة</v>
+      </c>
+      <c r="C43" t="str">
+        <v/>
+      </c>
+      <c r="D43" t="str">
+        <v>2026-02-12T00:00:00.000Z</v>
+      </c>
+      <c r="E43" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139008989
+Score: 35 | Recommendation: Ignore
+- No estimated value
+- 10 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F43">
+        <v>35</v>
+      </c>
+      <c r="G43" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H43" t="str">
+        <v>260139008989</v>
+      </c>
+      <c r="I43" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="44" xml:space="preserve">
+      <c r="A44" t="str">
+        <v>إدارة حوكمة أنظمة الوصول</v>
+      </c>
+      <c r="B44" t="str">
+        <v>مركز التأمين الصحي الوطني</v>
+      </c>
+      <c r="C44" t="str">
+        <v/>
+      </c>
+      <c r="D44" t="str">
+        <v>2026-02-09T00:00:00.000Z</v>
+      </c>
+      <c r="E44" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139007005
+Score: 34 | Recommendation: Ignore
+- No estimated value
+- 7 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F44">
+        <v>34</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H44" t="str">
+        <v>260139007005</v>
+      </c>
+      <c r="I44" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="45" xml:space="preserve">
+      <c r="A45" t="str">
+        <v>توريد وتركيب وتفعيل رخص البرامج الاحترافية</v>
+      </c>
+      <c r="B45" t="str">
+        <v>القوات الخاصة للأمن البيئي</v>
+      </c>
+      <c r="C45" t="str">
+        <v/>
+      </c>
+      <c r="D45" t="str">
+        <v>2026-02-08T00:00:00.000Z</v>
+      </c>
+      <c r="E45" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 251239008689
+Score: 33 | Recommendation: Ignore
+- No estimated value
+- 6 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F45">
+        <v>33</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H45" t="str">
+        <v>251239008689</v>
+      </c>
+      <c r="I45" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="46" xml:space="preserve">
+      <c r="A46" t="str">
+        <v>تجهيز ورش ومعامل المستقبل</v>
+      </c>
+      <c r="B46" t="str">
+        <v>جامعة حائل</v>
+      </c>
+      <c r="C46" t="str">
+        <v/>
+      </c>
+      <c r="D46" t="str">
+        <v>2026-02-07T00:00:00.000Z</v>
+      </c>
+      <c r="E46" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139005780
+Score: 33 | Recommendation: Ignore
+- No estimated value
+- 5 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F46">
+        <v>33</v>
+      </c>
+      <c r="G46" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H46" t="str">
+        <v>260139005780</v>
+      </c>
+      <c r="I46" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="47" xml:space="preserve">
+      <c r="A47" t="str">
+        <v>تطوير منصة التكامل المركزي للخدمات الرقمية</v>
+      </c>
+      <c r="B47" t="str">
+        <v>الهيئة العامة لعقارات الدولة</v>
+      </c>
+      <c r="C47" t="str">
+        <v/>
+      </c>
+      <c r="D47" t="str">
+        <v>2026-02-07T00:00:00.000Z</v>
+      </c>
+      <c r="E47" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139005930
+Score: 33 | Recommendation: Ignore
+- No estimated value
+- 5 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F47">
+        <v>33</v>
+      </c>
+      <c r="G47" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H47" t="str">
+        <v>260139005930</v>
+      </c>
+      <c r="I47" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="48" xml:space="preserve">
+      <c r="A48" t="str">
+        <v>تجديد رخص الخوادم VMware</v>
+      </c>
+      <c r="B48" t="str">
+        <v>مركز دعم اتخاذ القرار</v>
+      </c>
+      <c r="C48" t="str">
+        <v/>
+      </c>
+      <c r="D48" t="str">
+        <v>2026-02-07T00:00:00.000Z</v>
+      </c>
+      <c r="E48" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139006916
+Score: 33 | Recommendation: Ignore
+- No estimated value
+- 5 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F48">
+        <v>33</v>
+      </c>
+      <c r="G48" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H48" t="str">
+        <v>260139006916</v>
+      </c>
+      <c r="I48" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="49" xml:space="preserve">
+      <c r="A49" t="str">
+        <v>مشروع تشغيل وصيانة الحاسب الآلي (الخدمات المدارة )</v>
+      </c>
+      <c r="B49" t="str">
+        <v>أمارة منطقة جازان</v>
+      </c>
+      <c r="C49" t="str">
+        <v/>
+      </c>
+      <c r="D49" t="str">
+        <v>2026-02-05T00:00:00.000Z</v>
+      </c>
+      <c r="E49" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139000019
+Score: 32 | Recommendation: Ignore
+- No estimated value
+- 3 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F49">
+        <v>32</v>
+      </c>
+      <c r="G49" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H49" t="str">
+        <v>260139000019</v>
+      </c>
+      <c r="I49" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="50" xml:space="preserve">
+      <c r="A50" t="str">
+        <v>توفير دعم فني لمدة سنتين لنظام التواقيع الإلكترونية CodeTwo 365</v>
+      </c>
+      <c r="B50" t="str">
+        <v>الهيئة السعودية للمياه</v>
+      </c>
+      <c r="C50" t="str">
+        <v/>
+      </c>
+      <c r="D50" t="str">
+        <v>2026-02-05T00:00:00.000Z</v>
+      </c>
+      <c r="E50" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139005113
+Score: 32 | Recommendation: Ignore
+- No estimated value
+- 3 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F50">
+        <v>32</v>
+      </c>
+      <c r="G50" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H50" t="str">
+        <v>260139005113</v>
+      </c>
+      <c r="I50" t="str">
+        <v>etimad</v>
+      </c>
+    </row>
+    <row r="51" xml:space="preserve">
+      <c r="A51" t="str">
+        <v>تامين أجهزة اتصال مشفرة</v>
+      </c>
+      <c r="B51" t="str">
+        <v>وزارة التجارة</v>
+      </c>
+      <c r="C51" t="str">
+        <v/>
+      </c>
+      <c r="D51" t="str">
+        <v>2026-02-06T00:00:00.000Z</v>
+      </c>
+      <c r="E51" t="str" xml:space="preserve">
+        <v xml:space="preserve">Tender Number: 260139005916
+Score: 32 | Recommendation: Ignore
+- No estimated value
+- 4 days until deadline
+- Title and description present</v>
+      </c>
+      <c r="F51">
+        <v>32</v>
+      </c>
+      <c r="G51" t="str">
+        <v>Ignore</v>
+      </c>
+      <c r="H51" t="str">
+        <v>260139005916</v>
+      </c>
+      <c r="I51" t="str">
         <v>etimad</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I51"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>